<commit_message>
Inserita modifica komplett per non arrotondare ore modificate, inseriti metodi differenaziati per report pdf fidente, inserito arrotondamento per durata su ogni singola registrazione invece che sul giorno intero per fidente, rimosso flag direzione su txt app per le attività (creava problemi a komplett)
</commit_message>
<xml_diff>
--- a/PowerWeb/ExcelModels/ExportRegSemplice.xlsx
+++ b/PowerWeb/ExcelModels/ExportRegSemplice.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\PowerWebRepository\PowerWeb\PowerWeb\ExcelModels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\backup\PWNuovo\PowerWeb\ExcelModels\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D88673-DF5A-44DA-9B39-4F53B4290360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="135" windowWidth="17100" windowHeight="11385"/>
+    <workbookView xWindow="1050" yWindow="-120" windowWidth="27870" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Generale" sheetId="1" r:id="rId1"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
   <si>
     <t>COD. COLL.</t>
   </si>
@@ -54,17 +55,23 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[h]:mm:ss;@"/>
+    <numFmt numFmtId="166" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -122,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -131,9 +138,12 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -410,8 +420,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K10000"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N10000"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -421,12 +431,12 @@
     <col min="5" max="5" width="10.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="8.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.42578125" customWidth="1"/>
-    <col min="11" max="11" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="10.85546875" style="10" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -451,101 +461,111 @@
       <c r="H1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I2" s="9"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>

</xml_diff>